<commit_message>
Module 1 and 2 Fully Integrated
</commit_message>
<xml_diff>
--- a/data/module-4/dictionary.xlsx
+++ b/data/module-4/dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University Files\4th year\Research\Brahmi-Inscription-Translation\data\module-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3178E4A1-5544-4713-9D27-AEA8EC068CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F734B5E7-65C2-41E2-8C50-C7346FB06ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="577">
   <si>
     <t>Brhami Word</t>
   </si>
@@ -1736,9 +1736,6 @@
   </si>
   <si>
     <t>නන්ද</t>
-  </si>
-  <si>
-    <t>ප්‍රධනියා</t>
   </si>
   <si>
     <t>චතුදිශ</t>
@@ -2139,7 +2136,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L326"/>
+  <dimension ref="A1:B326"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="3"/>
@@ -2702,7 +2699,7 @@
         <v>125</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
@@ -3425,7 +3422,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A161" s="3" t="s">
         <v>296</v>
       </c>
@@ -3433,7 +3430,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
         <v>297</v>
       </c>
@@ -3441,7 +3438,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A163" s="3" t="s">
         <v>298</v>
       </c>
@@ -3449,7 +3446,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A164" s="3" t="s">
         <v>299</v>
       </c>
@@ -3457,15 +3454,15 @@
         <v>292</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A165" s="3" t="s">
         <v>300</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A166" s="3" t="s">
         <v>301</v>
       </c>
@@ -3473,7 +3470,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A167" s="3" t="s">
         <v>303</v>
       </c>
@@ -3481,7 +3478,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A168" s="3" t="s">
         <v>305</v>
       </c>
@@ -3489,7 +3486,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A169" s="3" t="s">
         <v>307</v>
       </c>
@@ -3497,7 +3494,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A170" s="3" t="s">
         <v>309</v>
       </c>
@@ -3505,7 +3502,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A171" s="3" t="s">
         <v>310</v>
       </c>
@@ -3513,7 +3510,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A172" s="3" t="s">
         <v>312</v>
       </c>
@@ -3521,18 +3518,15 @@
         <v>229</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A173" s="3" t="s">
         <v>313</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="L173" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A174" s="3" t="s">
         <v>315</v>
       </c>
@@ -3540,7 +3534,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A175" s="3" t="s">
         <v>317</v>
       </c>
@@ -3548,12 +3542,12 @@
         <v>318</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A176" s="3" t="s">
         <v>319</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>572</v>
+        <v>327</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.3">
@@ -4734,7 +4728,7 @@
     </row>
     <row r="324" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A324" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B324" s="3" t="s">
         <v>566</v>
@@ -4745,7 +4739,7 @@
         <v>330</v>
       </c>
       <c r="B325" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="326" spans="1:2" x14ac:dyDescent="0.3">
@@ -4753,7 +4747,7 @@
         <v>48</v>
       </c>
       <c r="B326" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>